<commit_message>
Benchmark: Good. LBracket: OK.
</commit_message>
<xml_diff>
--- a/data/LBracketDatabase.xlsx
+++ b/data/LBracketDatabase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Personal\suresh\Software\Github\ERSL-Private\METALS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C71ED06-164C-450B-89B8-7C93C921B0D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7ED2E1-CB60-4144-A4E2-C21182F9200A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2964" yWindow="2964" windowWidth="17280" windowHeight="8880" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="1" r:id="rId1"/>
@@ -25,34 +25,31 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t>Material</t>
+    <t>A</t>
   </si>
   <si>
-    <t>Elastic Modulus (Pa)</t>
+    <t>B</t>
   </si>
   <si>
-    <t>Yield Strength (Pa)</t>
+    <t>C</t>
   </si>
   <si>
-    <t>Density (kg/m^3)</t>
+    <t>E</t>
   </si>
   <si>
-    <t>In718</t>
+    <t>Y</t>
   </si>
   <si>
-    <t>Al6061</t>
-  </si>
-  <si>
-    <t>SS316</t>
+    <t>r</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -73,6 +70,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Symbol"/>
+      <family val="1"/>
+      <charset val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -110,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -122,6 +127,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -441,66 +452,64 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="2" max="2" width="22.21875" customWidth="1"/>
-    <col min="3" max="3" width="21.44140625" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="7.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="2"/>
+      <c r="B1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="4">
-        <v>2700</v>
-      </c>
-      <c r="C2" s="4">
-        <v>69000000000</v>
-      </c>
-      <c r="D2" s="4">
-        <v>275000000</v>
+        <v>0</v>
+      </c>
+      <c r="B2" s="5">
+        <v>0.27</v>
+      </c>
+      <c r="C2" s="5">
+        <v>0.6</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4">
-        <v>7850</v>
-      </c>
-      <c r="C3" s="4">
-        <v>210000000000</v>
-      </c>
-      <c r="D3" s="4">
-        <v>450000000</v>
+        <v>1</v>
+      </c>
+      <c r="B3" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="C3" s="5">
+        <v>0.92</v>
+      </c>
+      <c r="D3" s="5">
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="4">
-        <v>8192</v>
-      </c>
-      <c r="C4" s="4">
-        <v>200000000000</v>
-      </c>
-      <c r="D4" s="4">
-        <v>1000000000</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="5">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>